<commit_message>
Update Bra NPS By Segment reference file
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00 Reference Documents/Bra NPS By Segment.xlsx
+++ b/00 Reference Documents/Bra NPS By Segment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/KRBWEST/Documents/00 Intimo/01 Strategy/GPT Training/Original Algorithm/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/KRBWEST/Documents/00 Intimo/00 Claude Code/07 Fitme Algorithym/00 Reference Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B6E25607-8E9A-4745-BEA7-61BC539DE2E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05C728CE-12ED-A940-B9AB-FDFC74F24D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="46100" yWindow="500" windowWidth="22920" windowHeight="27020" xr2:uid="{4E3E5D8D-473B-9C47-ABEB-F7FDA6673888}"/>
+    <workbookView xWindow="5980" yWindow="760" windowWidth="22920" windowHeight="21580" xr2:uid="{4E3E5D8D-473B-9C47-ABEB-F7FDA6673888}"/>
   </bookViews>
   <sheets>
     <sheet name="Bra NPS by Style" sheetId="1" r:id="rId1"/>
@@ -328,6 +328,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Bra Selection"/>
@@ -9589,6 +9590,9 @@
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Bra Selection"/>
       <sheetName val="Style Price"/>
@@ -10196,6 +10200,7 @@
   <dimension ref="A1:J379"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="3" max="3" width="14.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.33203125" customWidth="1"/>
     <col min="6" max="6" width="11.83203125" style="2" customWidth="1"/>
     <col min="7" max="7" width="10.1640625" style="2" customWidth="1"/>

</xml_diff>